<commit_message>
feat(treet): complete Weeping Willow and custom tree generation
</commit_message>
<xml_diff>
--- a/RealMaxxin_Organization.xlsx
+++ b/RealMaxxin_Organization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GoldenGriffinGames\Projects\GoldenGriffinModding\Minecraft\Realmaxxin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A69485B-3D08-4147-AD0C-0885B227F9AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9788AF5-AF19-46E5-855A-CCC81526A867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Groups" sheetId="1" r:id="rId1"/>
@@ -585,15 +585,9 @@
     <t>Add more trees to the game in the form of fruit/nut growing varieties.</t>
   </si>
   <si>
-    <t>Food &amp; Processing</t>
-  </si>
-  <si>
     <t>Food and Processing</t>
   </si>
   <si>
-    <t>Adds more food recipes to the game for new fruits, vegetables, etc</t>
-  </si>
-  <si>
     <t>Machinery &amp; processing equipment</t>
   </si>
   <si>
@@ -757,6 +751,12 @@
   </si>
   <si>
     <t>Switches the drop for harvesting melons to a full melon. Rename vanilla “Melon” content to Watermelon where practical; preserve compatibility with vanilla IDs/tags.</t>
+  </si>
+  <si>
+    <t>Adds realistic food preparation, cooking, preservation and food-processing systems, from manual kitchen and butchery tasks to industrial production.</t>
+  </si>
+  <si>
+    <t>Hot Potato</t>
   </si>
 </sst>
 </file>
@@ -1260,33 +1260,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1301,6 +1274,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3599,202 +3599,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
     </row>
     <row r="3" spans="1:8" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="61"/>
+      <c r="G5" s="61"/>
+      <c r="H5" s="61"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
+      <c r="B6" s="61"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="61"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="57" t="s">
+      <c r="A7" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="57"/>
-      <c r="C7" s="57"/>
-      <c r="D7" s="57"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="61"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="57"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="57"/>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="57"/>
+      <c r="B9" s="61"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
+      <c r="B10" s="61"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="60"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
+      <c r="A11" s="65"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="60" t="s">
+      <c r="A12" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
+      <c r="B12" s="65"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="61"/>
-      <c r="B13" s="61"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="61"/>
+      <c r="A13" s="66"/>
+      <c r="B13" s="66"/>
+      <c r="C13" s="66"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="66"/>
+      <c r="F13" s="66"/>
+      <c r="G13" s="66"/>
+      <c r="H13" s="66"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="57" t="s">
+      <c r="A14" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="58" t="s">
+      <c r="A15" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="58"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="58"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="s">
+      <c r="A16" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
+      <c r="B16" s="67"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="67"/>
+      <c r="H16" s="67"/>
     </row>
     <row r="17" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="56" t="s">
+      <c r="A17" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="56"/>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
+      <c r="B17" s="63"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -4057,7 +4057,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="43" t="str">
-        <v>Food &amp; Processing</v>
+        <v>Hot Potato</v>
       </c>
       <c r="B27" s="9" t="str">
         <v>Agricrafture</v>
@@ -4078,7 +4078,7 @@
         <v>TBD</v>
       </c>
       <c r="H27" s="26" t="str">
-        <v>Adds more food recipes to the game for new fruits, vegetables, etc</v>
+        <v>Adds realistic food preparation, cooking, preservation and food-processing systems, from manual kitchen and butchery tasks to industrial production.</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -5093,6 +5093,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A17:H17"/>
@@ -5105,11 +5110,6 @@
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5198,43 +5198,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" spans="1:9" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
     </row>
     <row r="3" spans="1:9" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="63" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -5262,7 +5262,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="50" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C6" s="47" t="s">
         <v>25</v>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="E6" s="47"/>
       <c r="F6" s="40" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,7 +5280,7 @@
         <v>25</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C7" s="47" t="s">
         <v>21</v>
@@ -5290,7 +5290,7 @@
       </c>
       <c r="E7" s="47"/>
       <c r="F7" s="40" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -5298,7 +5298,7 @@
         <v>21</v>
       </c>
       <c r="B8" s="50" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C8" s="47" t="s">
         <v>24</v>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="E8" s="47"/>
       <c r="F8" s="40" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -5406,17 +5406,17 @@
         <v>26</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C14" s="48" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="48" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E14" s="48"/>
       <c r="F14" s="46" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -5424,17 +5424,17 @@
         <v>26</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C15" s="48" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="48" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E15" s="48"/>
       <c r="F15" s="46" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -5442,17 +5442,17 @@
         <v>26</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C16" s="48" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="48" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E16" s="48"/>
       <c r="F16" s="46" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -5460,7 +5460,7 @@
         <v>24</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C17" s="48" t="s">
         <v>23</v>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="E17" s="48"/>
       <c r="F17" s="46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -5478,7 +5478,7 @@
         <v>21</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C18" s="48" t="s">
         <v>26</v>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="E18" s="46"/>
       <c r="F18" s="46" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -5496,7 +5496,7 @@
         <v>21</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C19" s="48" t="s">
         <v>22</v>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="E19" s="46"/>
       <c r="F19" s="46" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -5514,17 +5514,17 @@
         <v>21</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C20" s="48" t="s">
         <v>23</v>
       </c>
       <c r="D20" s="48" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E20" s="46"/>
       <c r="F20" s="46" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -5532,17 +5532,17 @@
         <v>25</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C21" s="48" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="48" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E21" s="46"/>
       <c r="F21" s="46" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -5550,17 +5550,17 @@
         <v>26</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C22" s="48" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="48" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E22" s="46"/>
       <c r="F22" s="46" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -5568,17 +5568,17 @@
         <v>25</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C23" s="48" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="48" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E23" s="46"/>
       <c r="F23" s="46" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -9066,26 +9066,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -9151,12 +9151,12 @@
         <v>102</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>49</v>
@@ -9174,12 +9174,12 @@
         <v>102</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>51</v>
@@ -9197,7 +9197,7 @@
         <v>102</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -9287,11 +9287,11 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>145</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>30</v>
@@ -9304,12 +9304,12 @@
         <v>102</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>146</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>50</v>
@@ -9325,12 +9325,12 @@
         <v>102</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="43" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>47</v>
@@ -9346,15 +9346,15 @@
         <v>102</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="42" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>31</v>
@@ -9369,15 +9369,15 @@
         <v>102</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="43" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>31</v>
@@ -9392,7 +9392,7 @@
         <v>102</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -9625,26 +9625,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10146,26 +10146,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10608,26 +10608,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10666,7 +10666,7 @@
         <v>33</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F4" s="15" t="s">
         <v>102</v>
@@ -11087,26 +11087,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11132,11 +11132,11 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
-        <v>182</v>
+      <c r="A4" s="54" t="s">
+        <v>180</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>30</v>
@@ -11149,27 +11149,27 @@
         <v>102</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="67" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="64" t="s">
-        <v>183</v>
-      </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="58" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="55" t="s">
+        <v>181</v>
+      </c>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="66" t="s">
-        <v>195</v>
+      <c r="G5" s="57" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="43" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -11179,7 +11179,7 @@
         <v>102</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -11520,26 +11520,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11610,7 +11610,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -11621,7 +11621,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
@@ -11959,28 +11959,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">

</xml_diff>

<commit_message>
feat(treet): Add generic wooden furniture system with seating
</commit_message>
<xml_diff>
--- a/RealMaxxin_Organization.xlsx
+++ b/RealMaxxin_Organization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GoldenGriffinGames\Projects\GoldenGriffinModding\Minecraft\Realmaxxin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9788AF5-AF19-46E5-855A-CCC81526A867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507A9E03-764C-4F7D-825F-0087B060924E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Groups" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="208">
   <si>
     <t>And the umbrella name:</t>
   </si>
@@ -757,6 +757,24 @@
   </si>
   <si>
     <t>Hot Potato</t>
+  </si>
+  <si>
+    <t>Minecraft Mint</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Adds the ability to create coins and money with banner-style customization.  Could see it covering stuff like minted coins, denominations, maybe bullion or precious-metal processing, merchant/trading improvements, town economies, banking/storage, tolls/fees, payroll, vending-type machines, maybe even taxation or civic finance</t>
+  </si>
+  <si>
+    <t>Barges</t>
+  </si>
+  <si>
+    <t>Nauticrature / Constructure</t>
+  </si>
+  <si>
+    <t>Build various types of barges for different projects.</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1159,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1278,7 +1296,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1287,7 +1305,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1302,6 +1320,31 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
@@ -3611,28 +3654,28 @@
       <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
     </row>
     <row r="3" spans="1:8" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="64"/>
@@ -3785,16 +3828,16 @@
       <c r="H16" s="67"/>
     </row>
     <row r="17" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="63" t="s">
+      <c r="A17" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="63"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="63"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -3824,7 +3867,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="41" t="str" cm="1">
-        <f t="array" ref="A19:H57">_xlfn.LET(
+        <f t="array" ref="A19:H59">_xlfn.LET(
 _xlpm.clean,_xlfn.LAMBDA(_xlpm.t,IF(_xlpm.t="","",_xlpm.t)),
 _xlpm.addFamily,_xlfn.LAMBDA(_xlpm.t,_xlpm.f,
 _xlfn.LET(_xlpm.c,CLEAN(_xlpm.t),
@@ -4525,91 +4568,91 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="43" t="str">
-        <v>Resin-sealed Stone</v>
+        <v>Minecraft Mint</v>
       </c>
       <c r="B45" s="9" t="str">
-        <v>Constructure</v>
+        <v>Civicrafture</v>
       </c>
       <c r="C45" s="13" t="str">
-        <v>Materials</v>
+        <v>Economy</v>
       </c>
       <c r="D45" s="13" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="E45" s="13" t="str">
         <v>Idea</v>
       </c>
       <c r="F45" s="13" t="str">
-        <v>Tap Dancing</v>
+        <v/>
       </c>
       <c r="G45" s="13" t="str">
         <v>TBD</v>
       </c>
       <c r="H45" s="26" t="str">
-        <v>Keeps your Stone from turning to Cobblestone when you destroy it.</v>
+        <v>Adds the ability to create coins and money with banner-style customization.  Could see it covering stuff like minted coins, denominations, maybe bullion or precious-metal processing, merchant/trading improvements, town economies, banking/storage, tolls/fees, payroll, vending-type machines, maybe even taxation or civic finance</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="42" t="str">
-        <v>Staged Construction Sites</v>
+        <v>Resin-sealed Stone</v>
       </c>
       <c r="B46" s="24" t="str">
         <v>Constructure</v>
       </c>
       <c r="C46" s="19" t="str">
-        <v>Core Systems</v>
+        <v>Materials</v>
       </c>
       <c r="D46" s="19" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="E46" s="19" t="str">
-        <v>Planned</v>
+        <v>Idea</v>
       </c>
       <c r="F46" s="19" t="str">
-        <v>Blueprint System</v>
+        <v>Tap Dancing</v>
       </c>
       <c r="G46" s="19" t="str">
         <v>TBD</v>
       </c>
       <c r="H46" s="25" t="str">
-        <v>Large construction projects that require multiple stages and are not crafted like regular constructions.</v>
+        <v>Keeps your Stone from turning to Cobblestone when you destroy it.</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="43" t="str">
-        <v>Blueprint System</v>
+        <v>Staged Construction Sites</v>
       </c>
       <c r="B47" s="9" t="str">
         <v>Constructure</v>
       </c>
       <c r="C47" s="13" t="str">
-        <v>Planning</v>
+        <v>Core Systems</v>
       </c>
       <c r="D47" s="13" t="str">
-        <v>Low</v>
+        <v>High</v>
       </c>
       <c r="E47" s="13" t="str">
-        <v>Idea</v>
+        <v>Planned</v>
       </c>
       <c r="F47" s="13" t="str">
-        <v/>
+        <v>Blueprint System</v>
       </c>
       <c r="G47" s="13" t="str">
         <v>TBD</v>
       </c>
       <c r="H47" s="26" t="str">
-        <v>Places a project footprint and defines its construction stages and material requirements.</v>
+        <v>Large construction projects that require multiple stages and are not crafted like regular constructions.</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="42" t="str">
-        <v>Material Delivery to Construction Sites</v>
+        <v>Blueprint System</v>
       </c>
       <c r="B48" s="24" t="str">
         <v>Constructure</v>
       </c>
       <c r="C48" s="19" t="str">
-        <v>Logistics</v>
+        <v>Planning</v>
       </c>
       <c r="D48" s="19" t="str">
         <v>Low</v>
@@ -4618,56 +4661,56 @@
         <v>Idea</v>
       </c>
       <c r="F48" s="19" t="str">
-        <v>Staged Construction Sites</v>
+        <v/>
       </c>
       <c r="G48" s="19" t="str">
         <v>TBD</v>
       </c>
       <c r="H48" s="25" t="str">
-        <v>Have villagers able to bring materials to construction sites to help build them?</v>
+        <v>Places a project footprint and defines its construction stages and material requirements.</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="43" t="str">
-        <v>Flint Tools/Weapons</v>
+        <v>Material Delivery to Construction Sites</v>
       </c>
       <c r="B49" s="9" t="str">
         <v>Constructure</v>
       </c>
       <c r="C49" s="13" t="str">
-        <v>Weapons and Tools</v>
+        <v>Logistics</v>
       </c>
       <c r="D49" s="13" t="str">
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="E49" s="13" t="str">
-        <v>Modelling</v>
+        <v>Idea</v>
       </c>
       <c r="F49" s="13" t="str">
-        <v/>
+        <v>Staged Construction Sites</v>
       </c>
       <c r="G49" s="13" t="str">
         <v>TBD</v>
       </c>
       <c r="H49" s="26" t="str">
-        <v>Adds more uses for flint.</v>
+        <v>Have villagers able to bring materials to construction sites to help build them?</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="42" t="str">
-        <v>Herd Mentality</v>
+        <v>Flint Tools/Weapons</v>
       </c>
       <c r="B50" s="24" t="str">
-        <v>Faunacrafture</v>
+        <v>Constructure</v>
       </c>
       <c r="C50" s="19" t="str">
-        <v>Animal Husbandry</v>
+        <v>Weapons and Tools</v>
       </c>
       <c r="D50" s="19" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="E50" s="19" t="str">
-        <v>Idea</v>
+        <v>Modelling</v>
       </c>
       <c r="F50" s="19" t="str">
         <v/>
@@ -4676,24 +4719,24 @@
         <v>TBD</v>
       </c>
       <c r="H50" s="25" t="str">
-        <v>A proper breeding system with male and female animals, feeding troughs that can boost health/stats, bloodlines, diseases, food preferences, age/lifecycles, herd/flock behaviour, and more.</v>
+        <v>Adds more uses for flint.</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="43" t="str">
-        <v>Pasture &amp; Grazing System</v>
+        <v>Herd Mentality</v>
       </c>
       <c r="B51" s="9" t="str">
         <v>Faunacrafture</v>
       </c>
       <c r="C51" s="13" t="str">
-        <v/>
+        <v>Animal Husbandry</v>
       </c>
       <c r="D51" s="13" t="str">
-        <v/>
+        <v>Medium</v>
       </c>
       <c r="E51" s="13" t="str">
-        <v/>
+        <v>Idea</v>
       </c>
       <c r="F51" s="13" t="str">
         <v/>
@@ -4702,12 +4745,12 @@
         <v>TBD</v>
       </c>
       <c r="H51" s="26" t="str">
-        <v>Animals actually consume grass/forage, reduce pasture height, fertilise the ground, prefer certain forage, potentially damage overgrazed pasture, require supplemental feed when pasture is poor</v>
+        <v>A proper breeding system with male and female animals, feeding troughs that can boost health/stats, bloodlines, diseases, food preferences, age/lifecycles, herd/flock behaviour, and more.</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="42" t="str">
-        <v>Additional farm animals</v>
+        <v>Pasture &amp; Grazing System</v>
       </c>
       <c r="B52" s="24" t="str">
         <v>Faunacrafture</v>
@@ -4728,24 +4771,24 @@
         <v>TBD</v>
       </c>
       <c r="H52" s="25" t="str">
-        <v>Separate breeds of cows, sheep, pigs, chickens - new types of farm animals not included in Vanilla.</v>
+        <v>Animals actually consume grass/forage, reduce pasture height, fertilise the ground, prefer certain forage, potentially damage overgrazed pasture, require supplemental feed when pasture is poor</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="43" t="str">
-        <v>Oil &amp; Petroleum Industry</v>
+        <v>Additional farm animals</v>
       </c>
       <c r="B53" s="9" t="str">
-        <v>Mechanicrafture</v>
+        <v>Faunacrafture</v>
       </c>
       <c r="C53" s="13" t="str">
-        <v>Resources and Processing</v>
+        <v/>
       </c>
       <c r="D53" s="13" t="str">
-        <v>Medium</v>
+        <v/>
       </c>
       <c r="E53" s="13" t="str">
-        <v>Idea</v>
+        <v/>
       </c>
       <c r="F53" s="13" t="str">
         <v/>
@@ -4754,64 +4797,64 @@
         <v>TBD</v>
       </c>
       <c r="H53" s="26" t="str">
-        <v>Extract crude oil, refine it, and supply fuels/bitumen/lubricants across Realmaxxin’ mods.</v>
+        <v>Separate breeds of cows, sheep, pigs, chickens - new types of farm animals not included in Vanilla.</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="45" t="str">
-        <v>Plastics Industry</v>
+        <v>Oil &amp; Petroleum Industry</v>
       </c>
       <c r="B54" s="27" t="str">
         <v>Mechanicrafture</v>
       </c>
       <c r="C54" s="23" t="str">
-        <v>Materials &amp; Processing</v>
+        <v>Resources and Processing</v>
       </c>
       <c r="D54" s="23" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="E54" s="23" t="str">
         <v>Idea</v>
       </c>
       <c r="F54" s="23" t="str">
-        <v>Oil &amp; Petroleum Industry</v>
+        <v/>
       </c>
       <c r="G54" s="23" t="str">
         <v>TBD</v>
       </c>
       <c r="H54" s="28" t="str">
-        <v>Refine petroleum products into polymer pellets and manufactured plastic components used across Realmaxxin’.</v>
+        <v>Extract crude oil, refine it, and supply fuels/bitumen/lubricants across Realmaxxin’ mods.</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="43" t="str">
-        <v>Machinery &amp; Engines</v>
+        <v>Plastics Industry</v>
       </c>
       <c r="B55" s="9" t="str">
         <v>Mechanicrafture</v>
       </c>
       <c r="C55" s="13" t="str">
-        <v/>
+        <v>Materials &amp; Processing</v>
       </c>
       <c r="D55" s="13" t="str">
-        <v/>
+        <v>Low</v>
       </c>
       <c r="E55" s="13" t="str">
-        <v/>
+        <v>Idea</v>
       </c>
       <c r="F55" s="13" t="str">
-        <v/>
+        <v>Oil &amp; Petroleum Industry</v>
       </c>
       <c r="G55" s="13" t="str">
-        <v/>
+        <v>TBD</v>
       </c>
       <c r="H55" s="26" t="str">
-        <v/>
+        <v>Refine petroleum products into polymer pellets and manufactured plastic components used across Realmaxxin’.</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="45" t="str">
-        <v>Industrial Materials &amp; Processing</v>
+        <v>Machinery &amp; Engines</v>
       </c>
       <c r="B56" s="27" t="str">
         <v>Mechanicrafture</v>
@@ -4837,49 +4880,81 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="43" t="str">
+        <v>Industrial Materials &amp; Processing</v>
+      </c>
+      <c r="B57" s="9" t="str">
+        <v>Mechanicrafture</v>
+      </c>
+      <c r="C57" s="13" t="str">
+        <v/>
+      </c>
+      <c r="D57" s="13" t="str">
+        <v/>
+      </c>
+      <c r="E57" s="13" t="str">
+        <v/>
+      </c>
+      <c r="F57" s="13" t="str">
+        <v/>
+      </c>
+      <c r="G57" s="13" t="str">
+        <v/>
+      </c>
+      <c r="H57" s="26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="42" t="str">
         <v>Animal Water Transport</v>
       </c>
-      <c r="B57" s="9" t="str">
+      <c r="B58" s="24" t="str">
         <v>Faunacrafture / Nauticrafture</v>
       </c>
-      <c r="C57" s="13" t="str">
+      <c r="C58" s="19" t="str">
         <v>Transport</v>
       </c>
-      <c r="D57" s="13" t="str">
+      <c r="D58" s="19" t="str">
         <v>Low</v>
       </c>
-      <c r="E57" s="13" t="str">
+      <c r="E58" s="19" t="str">
         <v>Idea</v>
       </c>
-      <c r="F57" s="13" t="str">
+      <c r="F58" s="19" t="str">
         <v>Staged Construction Sites</v>
       </c>
-      <c r="G57" s="13" t="str">
+      <c r="G58" s="19" t="str">
         <v>TBD</v>
       </c>
-      <c r="H57" s="26" t="str">
+      <c r="H58" s="25" t="str">
         <v>A ship made to transport multiple animals at a time.</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="42"/>
-      <c r="B58" s="24"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="25"/>
-    </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="43"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="13"/>
-      <c r="H59" s="26"/>
+      <c r="A59" s="43" t="str">
+        <v>Barges</v>
+      </c>
+      <c r="B59" s="9" t="str">
+        <v>Nauticrature / Constructure</v>
+      </c>
+      <c r="C59" s="13" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="D59" s="13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E59" s="13" t="str">
+        <v>Idea</v>
+      </c>
+      <c r="F59" s="13" t="str">
+        <v>Staged Construction Sites</v>
+      </c>
+      <c r="G59" s="13" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="H59" s="26" t="str">
+        <v>Build various types of barges for different projects.</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="45"/>
@@ -5093,11 +5168,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A17:H17"/>
@@ -5110,6 +5180,11 @@
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5211,30 +5286,30 @@
       <c r="I1" s="59"/>
     </row>
     <row r="2" spans="1:9" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
     </row>
     <row r="3" spans="1:9" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -9077,15 +9152,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -9636,15 +9711,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10140,9 +10215,13 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.85546875" customWidth="1"/>
-    <col min="2" max="6" width="21.7109375" customWidth="1"/>
-    <col min="7" max="7" width="85.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="7" width="158.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
@@ -10157,15 +10236,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10191,101 +10270,113 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="70" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19" t="s">
+      <c r="E5" s="56"/>
+      <c r="F5" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="71" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="72" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="73" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="55" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="56" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19" t="s">
+      <c r="E7" s="56"/>
+      <c r="F7" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="71" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="10"/>
+    <row r="8" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="74" t="s">
+        <v>202</v>
+      </c>
+      <c r="B8" s="69" t="s">
+        <v>203</v>
+      </c>
+      <c r="C8" s="69" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="69"/>
+      <c r="F8" s="69" t="s">
+        <v>102</v>
+      </c>
+      <c r="G8" s="75" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
@@ -10619,15 +10710,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11098,15 +11189,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11531,15 +11622,15 @@
       <c r="G1" s="59"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11971,16 +12062,16 @@
       <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
@@ -12035,20 +12126,38 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="37"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="18"/>
+      <c r="A5" s="76" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="31"/>
       <c r="B6" s="38"/>
       <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="D6" s="13" t="s">
+        <v>29</v>
+      </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>

</xml_diff>

<commit_message>
feat(treet): implement Jurupa Oak worldgen and completed texture set
</commit_message>
<xml_diff>
--- a/RealMaxxin_Organization.xlsx
+++ b/RealMaxxin_Organization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GoldenGriffinGames\Projects\GoldenGriffinModding\Minecraft\Realmaxxin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{507A9E03-764C-4F7D-825F-0087B060924E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D60F34-812B-46E7-87B6-43136C386998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2250" yWindow="2070" windowWidth="21600" windowHeight="11385" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Groups" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="213">
   <si>
     <t>And the umbrella name:</t>
   </si>
@@ -775,6 +775,21 @@
   </si>
   <si>
     <t>Build various types of barges for different projects.</t>
+  </si>
+  <si>
+    <t>Explosives/Quarry Blasting</t>
+  </si>
+  <si>
+    <t>Mechanicrafture / Constructure</t>
+  </si>
+  <si>
+    <t>Mining</t>
+  </si>
+  <si>
+    <t>New Tools</t>
+  </si>
+  <si>
+    <t>Adds Large Pickaxe, Sledgehammer, Jackhammer, etc</t>
   </si>
 </sst>
 </file>
@@ -1293,33 +1308,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1345,6 +1333,33 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="3" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
@@ -1354,300 +1369,6 @@
     <cellStyle name="Title" xfId="1" builtinId="15"/>
   </cellStyles>
   <dxfs count="71">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="3"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3244,6 +2965,300 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="3"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3258,113 +3273,113 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16222BAD-9A18-4F16-9F55-73B87FCD0085}" name="tblAgricrafture" displayName="tblAgricrafture" ref="A3:G37" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69" tableBorderDxfId="68" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16222BAD-9A18-4F16-9F55-73B87FCD0085}" name="tblAgricrafture" displayName="tblAgricrafture" ref="A3:G37" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58" tableBorderDxfId="57" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G37" xr:uid="{16222BAD-9A18-4F16-9F55-73B87FCD0085}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{AFAFFEA5-6BAB-497B-9232-19AF2571115A}" name="Idea / Feature" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{0294D2B1-42AE-4EDF-9528-3596393D5870}" name="Category" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{CB8FEE43-B83F-4734-8D5C-D4464D421376}" name="Priority" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{DA1D7000-3470-485A-8C76-C29BDD30A34A}" name="Status" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{93DA2940-25CA-438B-983B-B7F821DA5187}" name="Dependencies" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{E89B0A38-0BF8-44C6-A2CB-69728CF6A201}" name="Target Release" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{85AB0DFB-04BA-4C69-A026-DACD2F7637C3}" name="Notes" dataDxfId="61"/>
+    <tableColumn id="1" xr3:uid="{AFAFFEA5-6BAB-497B-9232-19AF2571115A}" name="Idea / Feature" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{0294D2B1-42AE-4EDF-9528-3596393D5870}" name="Category" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{CB8FEE43-B83F-4734-8D5C-D4464D421376}" name="Priority" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{DA1D7000-3470-485A-8C76-C29BDD30A34A}" name="Status" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{93DA2940-25CA-438B-983B-B7F821DA5187}" name="Dependencies" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{E89B0A38-0BF8-44C6-A2CB-69728CF6A201}" name="Target Release" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{85AB0DFB-04BA-4C69-A026-DACD2F7637C3}" name="Notes" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C8A90FDD-2D38-4724-9483-4D69139455CA}" name="tblNauticrafture" displayName="tblNauticrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59" tableBorderDxfId="58" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C8A90FDD-2D38-4724-9483-4D69139455CA}" name="tblNauticrafture" displayName="tblNauticrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48" tableBorderDxfId="47" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G39" xr:uid="{C8A90FDD-2D38-4724-9483-4D69139455CA}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{460F7418-200A-4728-AAAD-31E7DF9165F5}" name="Idea / Feature" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{D48B0CD1-4D14-4990-9AC8-7F03288CFEB0}" name="Category" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{23C69C35-288B-483C-929F-03D6C5ADA4B2}" name="Priority" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{8E9CCD2E-F6E0-473D-B0D2-8222F450EA20}" name="Status" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{E1D25BA9-20EE-43F7-ADED-A7B911378FDD}" name="Dependencies" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{3C2CC766-887F-4164-863C-3143383EFB2E}" name="Target Release" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{1DE97419-CF72-4772-B718-24F99ADE920C}" name="Notes" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{460F7418-200A-4728-AAAD-31E7DF9165F5}" name="Idea / Feature" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{D48B0CD1-4D14-4990-9AC8-7F03288CFEB0}" name="Category" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{23C69C35-288B-483C-929F-03D6C5ADA4B2}" name="Priority" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{8E9CCD2E-F6E0-473D-B0D2-8222F450EA20}" name="Status" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{E1D25BA9-20EE-43F7-ADED-A7B911378FDD}" name="Dependencies" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{3C2CC766-887F-4164-863C-3143383EFB2E}" name="Target Release" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{1DE97419-CF72-4772-B718-24F99ADE920C}" name="Notes" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{428A90CA-35AD-411F-80AD-AE4D8A4B7A1F}" name="tblCivicrafture" displayName="tblCivicrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49" tableBorderDxfId="48" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{428A90CA-35AD-411F-80AD-AE4D8A4B7A1F}" name="tblCivicrafture" displayName="tblCivicrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38" tableBorderDxfId="37" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G39" xr:uid="{428A90CA-35AD-411F-80AD-AE4D8A4B7A1F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1B37A759-F418-4A64-90A3-716478974F23}" name="Idea / Feature" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{67FE852A-3B6B-4073-8ADA-E07F64913B64}" name="Category" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{3D8F6D4E-2A4C-4A93-A719-DB0AA731714B}" name="Priority" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{9B83FA4F-71A3-49E6-BD0F-21D54119B572}" name="Status" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{E59D5B3F-93CD-470B-95FB-8FF72D0ECA2C}" name="Dependencies" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{586B5198-E9FB-4172-890B-0324BBA4072A}" name="Target Release" dataDxfId="42"/>
-    <tableColumn id="7" xr3:uid="{E99F3A75-6910-4C68-92CC-D3AA311D332A}" name="Notes" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{1B37A759-F418-4A64-90A3-716478974F23}" name="Idea / Feature" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{67FE852A-3B6B-4073-8ADA-E07F64913B64}" name="Category" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{3D8F6D4E-2A4C-4A93-A719-DB0AA731714B}" name="Priority" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{9B83FA4F-71A3-49E6-BD0F-21D54119B572}" name="Status" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{E59D5B3F-93CD-470B-95FB-8FF72D0ECA2C}" name="Dependencies" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{586B5198-E9FB-4172-890B-0324BBA4072A}" name="Target Release" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{E99F3A75-6910-4C68-92CC-D3AA311D332A}" name="Notes" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F97C9F33-C0CE-422E-960D-6E10181A76C3}" name="tblConstructure" displayName="tblConstructure" ref="A3:G39" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39" tableBorderDxfId="38" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F97C9F33-C0CE-422E-960D-6E10181A76C3}" name="tblConstructure" displayName="tblConstructure" ref="A3:G39" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" tableBorderDxfId="27" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G39" xr:uid="{F97C9F33-C0CE-422E-960D-6E10181A76C3}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4DA8FED0-8548-4E14-BB12-B0C54F80AE85}" name="Idea / Feature" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{EAF7011E-3299-4954-9398-14F98D8FCB47}" name="Category" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{E51D2799-62AF-4DD6-9541-6AEC83D47B4F}" name="Priority" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{6D9188A5-7C4B-479D-A630-D2D3F1B47E68}" name="Status" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{4A513601-5AA1-428C-BBAE-D8005C3C710A}" name="Dependencies" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{6B3D1E22-C79D-4009-A7CC-2516FAAB72C0}" name="Target Release" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{7112C7CD-F013-4D2F-81BD-309C38AA830C}" name="Notes" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{4DA8FED0-8548-4E14-BB12-B0C54F80AE85}" name="Idea / Feature" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{EAF7011E-3299-4954-9398-14F98D8FCB47}" name="Category" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{E51D2799-62AF-4DD6-9541-6AEC83D47B4F}" name="Priority" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{6D9188A5-7C4B-479D-A630-D2D3F1B47E68}" name="Status" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{4A513601-5AA1-428C-BBAE-D8005C3C710A}" name="Dependencies" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{6B3D1E22-C79D-4009-A7CC-2516FAAB72C0}" name="Target Release" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{7112C7CD-F013-4D2F-81BD-309C38AA830C}" name="Notes" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C645CCBC-C365-4C9F-8756-AF8D8CA7180F}" name="tblFaunacrafture" displayName="tblFaunacrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29" tableBorderDxfId="28" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C645CCBC-C365-4C9F-8756-AF8D8CA7180F}" name="tblFaunacrafture" displayName="tblFaunacrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G39" xr:uid="{C645CCBC-C365-4C9F-8756-AF8D8CA7180F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4EA3AEA5-0E11-4557-8EB7-EAAE3705BCD9}" name="Idea / Feature" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{D8E827FC-0D68-4AF8-BE36-A86BBAB54530}" name="Category" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{F72FCC90-694D-4F24-983A-F3E44B1635B9}" name="Priority" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{160A73D8-C613-4104-8C17-9C51463650E8}" name="Status" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{222AF1A7-8AEC-439E-9AE8-C1496D4C3E25}" name="Dependencies" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{11FDAE28-F2CB-4CFF-9BAB-3532ADC0B0E0}" name="Target Release" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{09C05B12-490E-4AB1-BF56-3E9779F339FF}" name="Notes" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{4EA3AEA5-0E11-4557-8EB7-EAAE3705BCD9}" name="Idea / Feature" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{D8E827FC-0D68-4AF8-BE36-A86BBAB54530}" name="Category" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{F72FCC90-694D-4F24-983A-F3E44B1635B9}" name="Priority" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{160A73D8-C613-4104-8C17-9C51463650E8}" name="Status" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{222AF1A7-8AEC-439E-9AE8-C1496D4C3E25}" name="Dependencies" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{11FDAE28-F2CB-4CFF-9BAB-3532ADC0B0E0}" name="Target Release" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{09C05B12-490E-4AB1-BF56-3E9779F339FF}" name="Notes" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C7D7A416-0DD5-4FE9-9472-074AC22B370C}" name="tblMechanicrafture" displayName="tblMechanicrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C7D7A416-0DD5-4FE9-9472-074AC22B370C}" name="tblMechanicrafture" displayName="tblMechanicrafture" ref="A3:G39" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:G39" xr:uid="{C7D7A416-0DD5-4FE9-9472-074AC22B370C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{78177F67-8D8E-4BBC-B04A-364C005B96DD}" name="Idea / Feature" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{982B180E-0E93-4D22-9836-9DAF0DA9CE00}" name="Category" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{AA250904-4BF5-4114-A3EA-87B446D6B947}" name="Priority" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{E26FB936-C285-4DEF-AC1B-E4980F8F5D04}" name="Status" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{3988F212-E4F7-43B2-9F11-F0D1FE6E2584}" name="Dependencies" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{1FB6A337-09D8-476F-A6D1-BA57A1799D23}" name="Target Release" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{B72E350B-0342-4846-90A5-FE1C44E3FB4E}" name="Notes" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{78177F67-8D8E-4BBC-B04A-364C005B96DD}" name="Idea / Feature" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{982B180E-0E93-4D22-9836-9DAF0DA9CE00}" name="Category" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{AA250904-4BF5-4114-A3EA-87B446D6B947}" name="Priority" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{E26FB936-C285-4DEF-AC1B-E4980F8F5D04}" name="Status" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{3988F212-E4F7-43B2-9F11-F0D1FE6E2584}" name="Dependencies" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{1FB6A337-09D8-476F-A6D1-BA57A1799D23}" name="Target Release" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{B72E350B-0342-4846-90A5-FE1C44E3FB4E}" name="Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0FDE7CB6-B004-483F-884B-14F1349A2E3A}" name="tblCrossMod" displayName="tblCrossMod" ref="A3:H39" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" tableBorderDxfId="8" headerRowCellStyle="Heading 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0FDE7CB6-B004-483F-884B-14F1349A2E3A}" name="tblCrossMod" displayName="tblCrossMod" ref="A3:H39" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69" tableBorderDxfId="68" headerRowCellStyle="Heading 3">
   <autoFilter ref="A3:H39" xr:uid="{0FDE7CB6-B004-483F-884B-14F1349A2E3A}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{8855BF7C-7301-4773-83A9-ED0B635B4B9A}" name="Idea / Feature" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{F47E1F1F-6C31-40AB-91EF-502D5B72701F}" name="Mod Families" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{07B62D1D-41F5-4E2A-9209-73C5D2D9617B}" name="Category" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{79C4C785-B209-4D19-8095-BFBD563ABE3E}" name="Priority" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{7198CDF9-AD5A-46F7-BFA3-ED700A080C90}" name="Status" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{6B9948E7-BB62-496B-BDC6-51F81D823A19}" name="Dependencies" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{BF52D15F-3EA7-422D-B94C-B6D7B62E71B1}" name="Target Release" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{0DF5439E-CDB3-42BD-8F89-8EEC4D3CC8B7}" name="Notes" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{8855BF7C-7301-4773-83A9-ED0B635B4B9A}" name="Idea / Feature" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{F47E1F1F-6C31-40AB-91EF-502D5B72701F}" name="Mod Families" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{07B62D1D-41F5-4E2A-9209-73C5D2D9617B}" name="Category" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{79C4C785-B209-4D19-8095-BFBD563ABE3E}" name="Priority" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{7198CDF9-AD5A-46F7-BFA3-ED700A080C90}" name="Status" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{6B9948E7-BB62-496B-BDC6-51F81D823A19}" name="Dependencies" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{BF52D15F-3EA7-422D-B94C-B6D7B62E71B1}" name="Target Release" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{0DF5439E-CDB3-42BD-8F89-8EEC4D3CC8B7}" name="Notes" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3642,202 +3657,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
     </row>
     <row r="3" spans="1:8" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="64"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
+      <c r="A4" s="73"/>
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
-      <c r="H5" s="61"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="71"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="61"/>
+      <c r="B6" s="71"/>
+      <c r="C6" s="71"/>
+      <c r="D6" s="71"/>
+      <c r="E6" s="71"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="71"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="71"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="71"/>
+      <c r="H8" s="71"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="61"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="71"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="61"/>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
+      <c r="B10" s="71"/>
+      <c r="C10" s="71"/>
+      <c r="D10" s="71"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="71"/>
+      <c r="G10" s="71"/>
+      <c r="H10" s="71"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="65"/>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
+      <c r="A11" s="74"/>
+      <c r="B11" s="74"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="65" t="s">
+      <c r="A12" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="66"/>
-      <c r="B13" s="66"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="66"/>
-      <c r="F13" s="66"/>
-      <c r="G13" s="66"/>
-      <c r="H13" s="66"/>
+      <c r="A13" s="75"/>
+      <c r="B13" s="75"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="75"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="75"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="75"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="61"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="71"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="62"/>
-      <c r="C15" s="62"/>
-      <c r="D15" s="62"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="62"/>
-      <c r="G15" s="62"/>
-      <c r="H15" s="62"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="72"/>
+      <c r="G15" s="72"/>
+      <c r="H15" s="72"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="67" t="s">
+      <c r="A16" s="76" t="s">
         <v>139</v>
       </c>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
+      <c r="B16" s="76"/>
+      <c r="C16" s="76"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="76"/>
     </row>
     <row r="17" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="60"/>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="70"/>
+      <c r="F17" s="70"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="70"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -3867,7 +3882,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="41" t="str" cm="1">
-        <f t="array" ref="A19:H59">_xlfn.LET(
+        <f t="array" ref="A19:H61">_xlfn.LET(
 _xlpm.clean,_xlfn.LAMBDA(_xlpm.t,IF(_xlpm.t="","",_xlpm.t)),
 _xlpm.addFamily,_xlfn.LAMBDA(_xlpm.t,_xlpm.f,
 _xlfn.LET(_xlpm.c,CLEAN(_xlpm.t),
@@ -4724,16 +4739,16 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="43" t="str">
-        <v>Herd Mentality</v>
+        <v>New Tools</v>
       </c>
       <c r="B51" s="9" t="str">
-        <v>Faunacrafture</v>
+        <v>Constructure</v>
       </c>
       <c r="C51" s="13" t="str">
-        <v>Animal Husbandry</v>
+        <v>Weapons and Tools</v>
       </c>
       <c r="D51" s="13" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="E51" s="13" t="str">
         <v>Idea</v>
@@ -4745,24 +4760,24 @@
         <v>TBD</v>
       </c>
       <c r="H51" s="26" t="str">
-        <v>A proper breeding system with male and female animals, feeding troughs that can boost health/stats, bloodlines, diseases, food preferences, age/lifecycles, herd/flock behaviour, and more.</v>
+        <v>Adds Large Pickaxe, Sledgehammer, Jackhammer, etc</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="42" t="str">
-        <v>Pasture &amp; Grazing System</v>
+        <v>Herd Mentality</v>
       </c>
       <c r="B52" s="24" t="str">
         <v>Faunacrafture</v>
       </c>
       <c r="C52" s="19" t="str">
-        <v/>
+        <v>Animal Husbandry</v>
       </c>
       <c r="D52" s="19" t="str">
-        <v/>
+        <v>Medium</v>
       </c>
       <c r="E52" s="19" t="str">
-        <v/>
+        <v>Idea</v>
       </c>
       <c r="F52" s="19" t="str">
         <v/>
@@ -4771,12 +4786,12 @@
         <v>TBD</v>
       </c>
       <c r="H52" s="25" t="str">
-        <v>Animals actually consume grass/forage, reduce pasture height, fertilise the ground, prefer certain forage, potentially damage overgrazed pasture, require supplemental feed when pasture is poor</v>
+        <v>A proper breeding system with male and female animals, feeding troughs that can boost health/stats, bloodlines, diseases, food preferences, age/lifecycles, herd/flock behaviour, and more.</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="43" t="str">
-        <v>Additional farm animals</v>
+        <v>Pasture &amp; Grazing System</v>
       </c>
       <c r="B53" s="9" t="str">
         <v>Faunacrafture</v>
@@ -4797,24 +4812,24 @@
         <v>TBD</v>
       </c>
       <c r="H53" s="26" t="str">
-        <v>Separate breeds of cows, sheep, pigs, chickens - new types of farm animals not included in Vanilla.</v>
+        <v>Animals actually consume grass/forage, reduce pasture height, fertilise the ground, prefer certain forage, potentially damage overgrazed pasture, require supplemental feed when pasture is poor</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="45" t="str">
-        <v>Oil &amp; Petroleum Industry</v>
+        <v>Additional farm animals</v>
       </c>
       <c r="B54" s="27" t="str">
-        <v>Mechanicrafture</v>
+        <v>Faunacrafture</v>
       </c>
       <c r="C54" s="23" t="str">
-        <v>Resources and Processing</v>
+        <v/>
       </c>
       <c r="D54" s="23" t="str">
-        <v>Medium</v>
+        <v/>
       </c>
       <c r="E54" s="23" t="str">
-        <v>Idea</v>
+        <v/>
       </c>
       <c r="F54" s="23" t="str">
         <v/>
@@ -4823,64 +4838,64 @@
         <v>TBD</v>
       </c>
       <c r="H54" s="28" t="str">
-        <v>Extract crude oil, refine it, and supply fuels/bitumen/lubricants across Realmaxxin’ mods.</v>
+        <v>Separate breeds of cows, sheep, pigs, chickens - new types of farm animals not included in Vanilla.</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="43" t="str">
-        <v>Plastics Industry</v>
+        <v>Oil &amp; Petroleum Industry</v>
       </c>
       <c r="B55" s="9" t="str">
         <v>Mechanicrafture</v>
       </c>
       <c r="C55" s="13" t="str">
-        <v>Materials &amp; Processing</v>
+        <v>Resources and Processing</v>
       </c>
       <c r="D55" s="13" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="E55" s="13" t="str">
         <v>Idea</v>
       </c>
       <c r="F55" s="13" t="str">
-        <v>Oil &amp; Petroleum Industry</v>
+        <v/>
       </c>
       <c r="G55" s="13" t="str">
         <v>TBD</v>
       </c>
       <c r="H55" s="26" t="str">
-        <v>Refine petroleum products into polymer pellets and manufactured plastic components used across Realmaxxin’.</v>
+        <v>Extract crude oil, refine it, and supply fuels/bitumen/lubricants across Realmaxxin’ mods.</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="45" t="str">
-        <v>Machinery &amp; Engines</v>
+        <v>Plastics Industry</v>
       </c>
       <c r="B56" s="27" t="str">
         <v>Mechanicrafture</v>
       </c>
       <c r="C56" s="23" t="str">
-        <v/>
+        <v>Materials &amp; Processing</v>
       </c>
       <c r="D56" s="23" t="str">
-        <v/>
+        <v>Low</v>
       </c>
       <c r="E56" s="23" t="str">
-        <v/>
+        <v>Idea</v>
       </c>
       <c r="F56" s="23" t="str">
-        <v/>
+        <v>Oil &amp; Petroleum Industry</v>
       </c>
       <c r="G56" s="23" t="str">
-        <v/>
+        <v>TBD</v>
       </c>
       <c r="H56" s="28" t="str">
-        <v/>
+        <v>Refine petroleum products into polymer pellets and manufactured plastic components used across Realmaxxin’.</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="43" t="str">
-        <v>Industrial Materials &amp; Processing</v>
+        <v>Machinery &amp; Engines</v>
       </c>
       <c r="B57" s="9" t="str">
         <v>Mechanicrafture</v>
@@ -4906,36 +4921,36 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="42" t="str">
-        <v>Animal Water Transport</v>
+        <v>Industrial Materials &amp; Processing</v>
       </c>
       <c r="B58" s="24" t="str">
-        <v>Faunacrafture / Nauticrafture</v>
+        <v>Mechanicrafture</v>
       </c>
       <c r="C58" s="19" t="str">
-        <v>Transport</v>
+        <v/>
       </c>
       <c r="D58" s="19" t="str">
-        <v>Low</v>
+        <v/>
       </c>
       <c r="E58" s="19" t="str">
-        <v>Idea</v>
+        <v/>
       </c>
       <c r="F58" s="19" t="str">
-        <v>Staged Construction Sites</v>
+        <v/>
       </c>
       <c r="G58" s="19" t="str">
-        <v>TBD</v>
+        <v/>
       </c>
       <c r="H58" s="25" t="str">
-        <v>A ship made to transport multiple animals at a time.</v>
+        <v/>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="43" t="str">
-        <v>Barges</v>
+        <v>Animal Water Transport</v>
       </c>
       <c r="B59" s="9" t="str">
-        <v>Nauticrature / Constructure</v>
+        <v>Faunacrafture / Nauticrafture</v>
       </c>
       <c r="C59" s="13" t="str">
         <v>Transport</v>
@@ -4953,28 +4968,60 @@
         <v>TBD</v>
       </c>
       <c r="H59" s="26" t="str">
+        <v>A ship made to transport multiple animals at a time.</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="45" t="str">
+        <v>Barges</v>
+      </c>
+      <c r="B60" s="27" t="str">
+        <v>Nauticrature / Constructure</v>
+      </c>
+      <c r="C60" s="23" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="D60" s="23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E60" s="23" t="str">
+        <v>Idea</v>
+      </c>
+      <c r="F60" s="23" t="str">
+        <v>Staged Construction Sites</v>
+      </c>
+      <c r="G60" s="23" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="H60" s="28" t="str">
         <v>Build various types of barges for different projects.</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="45"/>
-      <c r="B60" s="27"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
-      <c r="E60" s="23"/>
-      <c r="F60" s="23"/>
-      <c r="G60" s="23"/>
-      <c r="H60" s="28"/>
-    </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="43"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="13"/>
-      <c r="E61" s="13"/>
-      <c r="F61" s="13"/>
-      <c r="G61" s="13"/>
-      <c r="H61" s="11"/>
+      <c r="A61" s="43" t="str">
+        <v>Explosives/Quarry Blasting</v>
+      </c>
+      <c r="B61" s="9" t="str">
+        <v>Mechanicrafture / Constructure</v>
+      </c>
+      <c r="C61" s="13" t="str">
+        <v>Mining</v>
+      </c>
+      <c r="D61" s="13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E61" s="13" t="str">
+        <v>Idea</v>
+      </c>
+      <c r="F61" s="13" t="str">
+        <v/>
+      </c>
+      <c r="G61" s="13" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="H61" s="11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="42"/>
@@ -5273,43 +5320,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
     </row>
     <row r="2" spans="1:9" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
     </row>
     <row r="3" spans="1:9" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -9141,26 +9188,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -9700,26 +9747,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10225,26 +10272,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10270,25 +10317,25 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="69" t="s">
+      <c r="E4" s="60" t="s">
         <v>99</v>
       </c>
-      <c r="F4" s="69" t="s">
+      <c r="F4" s="60" t="s">
         <v>102</v>
       </c>
-      <c r="G4" s="70" t="s">
+      <c r="G4" s="61" t="s">
         <v>54</v>
       </c>
     </row>
@@ -10309,30 +10356,30 @@
       <c r="F5" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="71" t="s">
+      <c r="G5" s="62" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="72" t="s">
+      <c r="A6" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="69" t="s">
+      <c r="D6" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="69" t="s">
+      <c r="E6" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="69" t="s">
+      <c r="F6" s="60" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="73" t="s">
+      <c r="G6" s="64" t="s">
         <v>107</v>
       </c>
     </row>
@@ -10353,28 +10400,28 @@
       <c r="F7" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="G7" s="71" t="s">
+      <c r="G7" s="62" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="65" t="s">
         <v>202</v>
       </c>
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="60" t="s">
         <v>203</v>
       </c>
-      <c r="C8" s="69" t="s">
+      <c r="C8" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69" t="s">
+      <c r="E8" s="60"/>
+      <c r="F8" s="60" t="s">
         <v>102</v>
       </c>
-      <c r="G8" s="75" t="s">
+      <c r="G8" s="66" t="s">
         <v>204</v>
       </c>
     </row>
@@ -10699,26 +10746,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -10855,13 +10902,25 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="17"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
+      <c r="A9" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>33</v>
+      </c>
       <c r="E9" s="18"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="18"/>
+      <c r="F9" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="20"/>
@@ -11178,26 +11237,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -11611,26 +11670,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -12045,33 +12104,34 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
-    <col min="2" max="7" width="21.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" style="1" customWidth="1"/>
+    <col min="3" max="7" width="21.5703125" style="1" customWidth="1"/>
     <col min="8" max="8" width="85.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
     </row>
     <row r="2" spans="1:8" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
@@ -12126,7 +12186,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="67" t="s">
         <v>205</v>
       </c>
       <c r="B5" s="37" t="s">
@@ -12152,15 +12212,25 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="31"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="13"/>
+      <c r="A6" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>210</v>
+      </c>
       <c r="D6" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="13"/>
+      <c r="E6" s="13" t="s">
+        <v>33</v>
+      </c>
       <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
+      <c r="G6" s="13" t="s">
+        <v>102</v>
+      </c>
       <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>